<commit_message>
Added more training results
</commit_message>
<xml_diff>
--- a/train_results.xlsx
+++ b/train_results.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Train overview" sheetId="1" state="visible" r:id="rId2"/>
@@ -188,7 +188,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -201,7 +201,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -211,6 +211,10 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -231,7 +235,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.89"/>
   </cols>
@@ -539,7 +543,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.59"/>
   </cols>
@@ -739,7 +743,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.59"/>
   </cols>
@@ -925,7 +929,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.59"/>
   </cols>
@@ -1111,7 +1115,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.59"/>
   </cols>
@@ -1297,7 +1301,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.59"/>
   </cols>
@@ -1477,7 +1481,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K26"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1566,21 +1570,39 @@
       <c r="K4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
+      <c r="C5" s="6" t="n">
+        <v>17006</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>16994</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>2994</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>3006</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>64</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>0.503899073822701</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>73.81</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>84.93</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">

</xml_diff>

<commit_message>
Fixed bug where wrong trained model was being saved
</commit_message>
<xml_diff>
--- a/train_results.xlsx
+++ b/train_results.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Train overview" sheetId="1" state="visible" r:id="rId2"/>
@@ -188,7 +188,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -201,12 +201,16 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -235,7 +239,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.89"/>
   </cols>
@@ -397,132 +401,132 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="0" t="n">
+      <c r="C7" s="4" t="n">
         <v>16981</v>
       </c>
-      <c r="D7" s="0" t="n">
+      <c r="D7" s="4" t="n">
         <v>17019</v>
       </c>
-      <c r="E7" s="0" t="n">
+      <c r="E7" s="4" t="n">
         <v>3019</v>
       </c>
-      <c r="F7" s="0" t="n">
+      <c r="F7" s="4" t="n">
         <v>2981</v>
       </c>
-      <c r="G7" s="0" t="n">
+      <c r="G7" s="4" t="n">
         <v>0.502804518219024</v>
       </c>
-      <c r="H7" s="0" t="n">
+      <c r="H7" s="4" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="0" t="n">
+      <c r="C8" s="4" t="n">
         <v>16972</v>
       </c>
-      <c r="D8" s="0" t="n">
+      <c r="D8" s="4" t="n">
         <v>17028</v>
       </c>
-      <c r="E8" s="0" t="n">
+      <c r="E8" s="4" t="n">
         <v>3028</v>
       </c>
-      <c r="F8" s="0" t="n">
+      <c r="F8" s="4" t="n">
         <v>2972</v>
       </c>
-      <c r="G8" s="0" t="n">
+      <c r="G8" s="4" t="n">
         <v>0.502050775384146</v>
       </c>
-      <c r="H8" s="0" t="n">
+      <c r="H8" s="4" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="0" t="n">
+      <c r="C9" s="4" t="n">
         <v>16943</v>
       </c>
-      <c r="D9" s="0" t="n">
+      <c r="D9" s="4" t="n">
         <v>17057</v>
       </c>
-      <c r="E9" s="0" t="n">
+      <c r="E9" s="4" t="n">
         <v>3057</v>
       </c>
-      <c r="F9" s="0" t="n">
+      <c r="F9" s="4" t="n">
         <v>2943</v>
       </c>
-      <c r="G9" s="0" t="n">
+      <c r="G9" s="4" t="n">
         <v>0.500262489867589</v>
       </c>
-      <c r="H9" s="0" t="n">
+      <c r="H9" s="4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="0" t="n">
+      <c r="C10" s="4" t="n">
         <v>17030</v>
       </c>
-      <c r="D10" s="0" t="n">
+      <c r="D10" s="4" t="n">
         <v>16070</v>
       </c>
-      <c r="E10" s="0" t="n">
+      <c r="E10" s="4" t="n">
         <v>2970</v>
       </c>
-      <c r="F10" s="0" t="n">
+      <c r="F10" s="4" t="n">
         <v>3030</v>
       </c>
-      <c r="G10" s="0" t="n">
+      <c r="G10" s="4" t="n">
         <v>0.510409388277266</v>
       </c>
-      <c r="H10" s="0" t="n">
+      <c r="H10" s="4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="0" t="n">
+      <c r="C11" s="4" t="n">
         <v>16980</v>
       </c>
-      <c r="D11" s="0" t="n">
+      <c r="D11" s="4" t="n">
         <v>17020</v>
       </c>
-      <c r="E11" s="0" t="n">
+      <c r="E11" s="4" t="n">
         <v>3020</v>
       </c>
-      <c r="F11" s="0" t="n">
+      <c r="F11" s="4" t="n">
         <v>2980</v>
       </c>
-      <c r="G11" s="0" t="n">
+      <c r="G11" s="4" t="n">
         <v>0.506366344671401</v>
       </c>
-      <c r="H11" s="0" t="n">
+      <c r="H11" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -543,22 +547,22 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.59"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3" t="s">
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
@@ -625,7 +629,7 @@
       <c r="F4" s="2" t="n">
         <v>99.88</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="G4" s="3" t="n">
         <v>99.5</v>
       </c>
     </row>
@@ -639,7 +643,7 @@
       <c r="C5" s="2" t="n">
         <v>99.94</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="3" t="n">
         <v>88.3</v>
       </c>
       <c r="E5" s="2" t="n">
@@ -743,23 +747,23 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.59"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3" t="s">
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
@@ -803,7 +807,7 @@
       <c r="F3" s="2" t="n">
         <v>99.71</v>
       </c>
-      <c r="G3" s="4" t="n">
+      <c r="G3" s="3" t="n">
         <v>99.45</v>
       </c>
     </row>
@@ -840,7 +844,7 @@
       <c r="C5" s="2" t="n">
         <v>99.89</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="3" t="n">
         <v>85.65</v>
       </c>
       <c r="E5" s="2" t="n">
@@ -929,23 +933,23 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.59"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3" t="s">
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
@@ -989,7 +993,7 @@
       <c r="F3" s="2" t="n">
         <v>99.77</v>
       </c>
-      <c r="G3" s="4" t="n">
+      <c r="G3" s="3" t="n">
         <v>99.44</v>
       </c>
     </row>
@@ -1026,7 +1030,7 @@
       <c r="C5" s="2" t="n">
         <v>99.98</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="3" t="n">
         <v>83.05</v>
       </c>
       <c r="E5" s="2" t="n">
@@ -1115,23 +1119,23 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.59"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3" t="s">
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
@@ -1175,7 +1179,7 @@
       <c r="F3" s="2" t="n">
         <v>99.83</v>
       </c>
-      <c r="G3" s="4" t="n">
+      <c r="G3" s="3" t="n">
         <v>99.4</v>
       </c>
     </row>
@@ -1212,7 +1216,7 @@
       <c r="C5" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="3" t="n">
         <v>80.61</v>
       </c>
       <c r="E5" s="2" t="n">
@@ -1301,7 +1305,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.59"/>
   </cols>
@@ -1313,7 +1317,7 @@
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="6" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1359,7 +1363,7 @@
       <c r="F3" s="2" t="n">
         <v>99.83</v>
       </c>
-      <c r="G3" s="4" t="n">
+      <c r="G3" s="3" t="n">
         <v>99.34</v>
       </c>
     </row>
@@ -1396,7 +1400,7 @@
       <c r="C5" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="3" t="n">
         <v>77.77</v>
       </c>
       <c r="E5" s="2" t="n">
@@ -1481,7 +1485,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K26"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1570,37 +1574,37 @@
       <c r="K4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="C5" s="2" t="n">
         <v>17006</v>
       </c>
-      <c r="D5" s="6" t="n">
+      <c r="D5" s="2" t="n">
         <v>16994</v>
       </c>
-      <c r="E5" s="6" t="n">
+      <c r="E5" s="2" t="n">
         <v>2994</v>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="F5" s="2" t="n">
         <v>3006</v>
       </c>
-      <c r="G5" s="6" t="n">
+      <c r="G5" s="2" t="n">
         <v>64</v>
       </c>
-      <c r="H5" s="6" t="n">
+      <c r="H5" s="2" t="n">
         <v>0.503899073822701</v>
       </c>
-      <c r="I5" s="6" t="n">
+      <c r="I5" s="2" t="n">
         <v>73.81</v>
       </c>
-      <c r="J5" s="6" t="n">
+      <c r="J5" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="K5" s="6" t="n">
+      <c r="K5" s="2" t="n">
         <v>84.93</v>
       </c>
     </row>
@@ -1748,15 +1752,33 @@
       <c r="B13" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
+      <c r="C13" s="2" t="n">
+        <v>17031</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>16969</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>2969</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>3031</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>128</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>0.50509884430373</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>68.35</v>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="K13" s="2" t="n">
+        <v>81.2</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
@@ -1765,32 +1787,68 @@
       <c r="B14" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
+      <c r="C14" s="2" t="n">
+        <v>16950</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>17050</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>3050</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>2950</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>0.499920884503963</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>83.19</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="K14" s="2" t="n">
+        <v>90.83</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
-      <c r="J15" s="4"/>
-      <c r="K15" s="4"/>
+      <c r="C15" s="7" t="n">
+        <v>16957</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>17043</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>3043</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>2957</v>
+      </c>
+      <c r="G15" s="7" t="n">
+        <v>64</v>
+      </c>
+      <c r="H15" s="7" t="n">
+        <v>0.500362905416083</v>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>65.07</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>99.88</v>
+      </c>
+      <c r="K15" s="7" t="n">
+        <v>78.8</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
@@ -1799,15 +1857,33 @@
       <c r="B16" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
+      <c r="C16" s="2" t="n">
+        <v>17028</v>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>16972</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>2972</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>3028</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>0.505012486209261</v>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>67.54</v>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>99.89</v>
+      </c>
+      <c r="K16" s="2" t="n">
+        <v>80.59</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">

</xml_diff>

<commit_message>
Added updated results changed VGG model unfreeze
</commit_message>
<xml_diff>
--- a/train_results.xlsx
+++ b/train_results.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Train overview" sheetId="1" state="visible" r:id="rId2"/>
@@ -201,7 +201,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -223,14 +223,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -328,7 +320,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.89"/>
   </cols>
@@ -366,6 +358,24 @@
       <c r="B2" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="C2" s="0" t="n">
+        <v>16968</v>
+      </c>
+      <c r="D2" s="0" t="n">
+        <v>17032</v>
+      </c>
+      <c r="E2" s="0" t="n">
+        <v>3032</v>
+      </c>
+      <c r="F2" s="0" t="n">
+        <v>2968</v>
+      </c>
+      <c r="G2" s="0" t="n">
+        <v>0.502014754310487</v>
+      </c>
+      <c r="H2" s="0" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
@@ -374,6 +384,24 @@
       <c r="B3" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="C3" s="0" t="n">
+        <v>16978</v>
+      </c>
+      <c r="D3" s="0" t="n">
+        <v>17022</v>
+      </c>
+      <c r="E3" s="0" t="n">
+        <v>3022</v>
+      </c>
+      <c r="F3" s="0" t="n">
+        <v>2978</v>
+      </c>
+      <c r="G3" s="0" t="n">
+        <v>0.502216119141806</v>
+      </c>
+      <c r="H3" s="0" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
@@ -382,6 +410,24 @@
       <c r="B4" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="C4" s="0" t="n">
+        <v>16970</v>
+      </c>
+      <c r="D4" s="0" t="n">
+        <v>17030</v>
+      </c>
+      <c r="E4" s="0" t="n">
+        <v>3030</v>
+      </c>
+      <c r="F4" s="0" t="n">
+        <v>2970</v>
+      </c>
+      <c r="G4" s="0" t="n">
+        <v>0.501611094626169</v>
+      </c>
+      <c r="H4" s="0" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
@@ -390,6 +436,24 @@
       <c r="B5" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="C5" s="0" t="n">
+        <v>16989</v>
+      </c>
+      <c r="D5" s="0" t="n">
+        <v>17011</v>
+      </c>
+      <c r="E5" s="0" t="n">
+        <v>3011</v>
+      </c>
+      <c r="F5" s="0" t="n">
+        <v>2989</v>
+      </c>
+      <c r="G5" s="0" t="n">
+        <v>0.512986568704484</v>
+      </c>
+      <c r="H5" s="0" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
@@ -398,6 +462,24 @@
       <c r="B6" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="C6" s="0" t="n">
+        <v>16988</v>
+      </c>
+      <c r="D6" s="0" t="n">
+        <v>17012</v>
+      </c>
+      <c r="E6" s="0" t="n">
+        <v>3012</v>
+      </c>
+      <c r="F6" s="0" t="n">
+        <v>2988</v>
+      </c>
+      <c r="G6" s="0" t="n">
+        <v>0.514079347489372</v>
+      </c>
+      <c r="H6" s="0" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
@@ -406,12 +488,24 @@
       <c r="B7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
+      <c r="C7" s="4" t="n">
+        <v>17011</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>16989</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>2989</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>3011</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>0.504649150939215</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
@@ -486,7 +580,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.59"/>
   </cols>
@@ -530,31 +624,55 @@
       <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
+      <c r="B3" s="2" t="n">
+        <v>54.95</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>99.97</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>70.92</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>99.43</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>99.33</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>99.38</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
+      <c r="B4" s="2" t="n">
+        <v>65.77</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>99.91</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>79.32</v>
+      </c>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
-      <c r="G4" s="6"/>
+      <c r="G4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="6"/>
+      <c r="B5" s="2" t="n">
+        <v>86.52</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>99.71</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>92.65</v>
+      </c>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -563,9 +681,15 @@
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
+      <c r="B6" s="2" t="n">
+        <v>74.14</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>93.58</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>82.74</v>
+      </c>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
@@ -574,9 +698,15 @@
       <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
+      <c r="B7" s="2" t="n">
+        <v>72.49</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>93.44</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>81.65</v>
+      </c>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
@@ -626,7 +756,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.59"/>
   </cols>
@@ -671,56 +801,92 @@
       <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
+      <c r="B3" s="2" t="n">
+        <v>53.41</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>69.63</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>99.23</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>99.62</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>99.43</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
+      <c r="B4" s="2" t="n">
+        <v>65.32</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>99.91</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>78.99</v>
+      </c>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
+      <c r="B5" s="2" t="n">
+        <v>84.35</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>99.82</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>91.44</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
+      <c r="B6" s="2" t="n">
+        <v>65.4</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>96.5</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>77.96</v>
+      </c>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
+      <c r="B7" s="2" t="n">
+        <v>67.35</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>95.53</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2"/>
@@ -752,7 +918,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.59"/>
   </cols>
@@ -797,56 +963,92 @@
       <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
+      <c r="B3" s="2" t="n">
+        <v>52.07</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>68.48</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>98.96</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>99.79</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>99.37</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
+      <c r="B4" s="2" t="n">
+        <v>64.62</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>99.98</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>78.5</v>
+      </c>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
+      <c r="B5" s="2" t="n">
+        <v>82.65</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>99.82</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>90.43</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
+      <c r="B6" s="2" t="n">
+        <v>58.61</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>98.02</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>73.36</v>
+      </c>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
+      <c r="B7" s="2" t="n">
+        <v>62.94</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>97.02</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>76.34</v>
+      </c>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2"/>
@@ -878,7 +1080,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.59"/>
   </cols>
@@ -923,56 +1125,92 @@
       <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
+      <c r="B3" s="2" t="n">
+        <v>50.92</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>67.48</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>98.74</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>99.86</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>99.3</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
+      <c r="B4" s="2" t="n">
+        <v>64.08</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>99.98</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>78.1</v>
+      </c>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
+      <c r="B5" s="2" t="n">
+        <v>80.27</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>99.87</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
+      <c r="B6" s="2" t="n">
+        <v>53.54</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>98.92</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>69.48</v>
+      </c>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
+      <c r="B7" s="2" t="n">
+        <v>60.31</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>74.67</v>
+      </c>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2"/>
@@ -1004,23 +1242,23 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.59"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7" t="s">
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
@@ -1049,56 +1287,92 @@
       <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
+      <c r="B3" s="2" t="n">
+        <v>49.59</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>66.31</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>98.51</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>99.91</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>99.21</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
+      <c r="B4" s="2" t="n">
+        <v>63.07</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>77.35</v>
+      </c>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
+      <c r="B5" s="2" t="n">
+        <v>78.18</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>99.94</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>87.73</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
+      <c r="B6" s="2" t="n">
+        <v>49.65</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>99.34</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>66.21</v>
+      </c>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
+      <c r="B7" s="2" t="n">
+        <v>57.82</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>98.9</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>72.97</v>
+      </c>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2"/>
@@ -1130,40 +1404,40 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K26"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="G1" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="H1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="I1" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="J1" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="K1" s="8" t="s">
+      <c r="K1" s="6" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1236,106 +1510,106 @@
       <c r="K5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="9"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="7"/>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="10"/>
-      <c r="H7" s="10"/>
-      <c r="I7" s="10"/>
-      <c r="J7" s="10"/>
-      <c r="K7" s="10"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
-      <c r="K8" s="10"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="10"/>
-      <c r="I9" s="10"/>
-      <c r="J9" s="10"/>
-      <c r="K9" s="10"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="10"/>
-      <c r="H10" s="10"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
-      <c r="K10" s="10"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="8"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="11"/>
-      <c r="J11" s="11"/>
-      <c r="K11" s="11"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="9"/>
+      <c r="J11" s="9"/>
+      <c r="K11" s="9"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
@@ -1406,106 +1680,106 @@
       <c r="K15" s="2"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9" t="s">
+      <c r="A16" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="9"/>
-      <c r="I16" s="9"/>
-      <c r="J16" s="9"/>
-      <c r="K16" s="9"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="7"/>
+      <c r="I16" s="7"/>
+      <c r="J16" s="7"/>
+      <c r="K16" s="7"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10" t="s">
+      <c r="A17" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="10"/>
-      <c r="J17" s="10"/>
-      <c r="K17" s="10"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
+      <c r="K17" s="8"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="s">
+      <c r="A18" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="10"/>
-      <c r="H18" s="10"/>
-      <c r="I18" s="10"/>
-      <c r="J18" s="10"/>
-      <c r="K18" s="10"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="8"/>
+      <c r="K18" s="8"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10" t="s">
+      <c r="A19" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="10"/>
-      <c r="H19" s="10"/>
-      <c r="I19" s="10"/>
-      <c r="J19" s="10"/>
-      <c r="K19" s="10"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="8"/>
+      <c r="J19" s="8"/>
+      <c r="K19" s="8"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="10"/>
-      <c r="H20" s="10"/>
-      <c r="I20" s="10"/>
-      <c r="J20" s="10"/>
-      <c r="K20" s="10"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
+      <c r="I20" s="8"/>
+      <c r="J20" s="8"/>
+      <c r="K20" s="8"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
+      <c r="A21" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B21" s="11" t="s">
+      <c r="B21" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="11"/>
-      <c r="J21" s="11"/>
-      <c r="K21" s="11"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
+      <c r="J21" s="9"/>
+      <c r="K21" s="9"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
@@ -1576,21 +1850,21 @@
       <c r="K25" s="2"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="9" t="s">
+      <c r="A26" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="B26" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="9"/>
-      <c r="H26" s="9"/>
-      <c r="I26" s="9"/>
-      <c r="J26" s="9"/>
-      <c r="K26" s="9"/>
+      <c r="C26" s="7"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7"/>
+      <c r="F26" s="7"/>
+      <c r="G26" s="7"/>
+      <c r="H26" s="7"/>
+      <c r="I26" s="7"/>
+      <c r="J26" s="7"/>
+      <c r="K26" s="7"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Removed old incorrect results
</commit_message>
<xml_diff>
--- a/train_results.xlsx
+++ b/train_results.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Train overview" sheetId="1" state="visible" r:id="rId2"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="25">
   <si>
     <t xml:space="preserve">Model</t>
   </si>
@@ -86,9 +86,6 @@
   </si>
   <si>
     <t xml:space="preserve">F1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">99l.53</t>
   </si>
   <si>
     <t xml:space="preserve">valid+</t>
@@ -323,7 +320,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.89"/>
   </cols>
@@ -361,24 +358,6 @@
       <c r="B2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="0" t="n">
-        <v>16968</v>
-      </c>
-      <c r="D2" s="0" t="n">
-        <v>17032</v>
-      </c>
-      <c r="E2" s="0" t="n">
-        <v>3032</v>
-      </c>
-      <c r="F2" s="0" t="n">
-        <v>2968</v>
-      </c>
-      <c r="G2" s="0" t="n">
-        <v>0.502014754310487</v>
-      </c>
-      <c r="H2" s="0" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
@@ -387,24 +366,6 @@
       <c r="B3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="0" t="n">
-        <v>16978</v>
-      </c>
-      <c r="D3" s="0" t="n">
-        <v>17022</v>
-      </c>
-      <c r="E3" s="0" t="n">
-        <v>3022</v>
-      </c>
-      <c r="F3" s="0" t="n">
-        <v>2978</v>
-      </c>
-      <c r="G3" s="0" t="n">
-        <v>0.502216119141806</v>
-      </c>
-      <c r="H3" s="0" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
@@ -413,24 +374,6 @@
       <c r="B4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="0" t="n">
-        <v>16970</v>
-      </c>
-      <c r="D4" s="0" t="n">
-        <v>17030</v>
-      </c>
-      <c r="E4" s="0" t="n">
-        <v>3030</v>
-      </c>
-      <c r="F4" s="0" t="n">
-        <v>2970</v>
-      </c>
-      <c r="G4" s="0" t="n">
-        <v>0.501611094626169</v>
-      </c>
-      <c r="H4" s="0" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
@@ -439,24 +382,6 @@
       <c r="B5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="0" t="n">
-        <v>16989</v>
-      </c>
-      <c r="D5" s="0" t="n">
-        <v>17011</v>
-      </c>
-      <c r="E5" s="0" t="n">
-        <v>3011</v>
-      </c>
-      <c r="F5" s="0" t="n">
-        <v>2989</v>
-      </c>
-      <c r="G5" s="0" t="n">
-        <v>0.512986568704484</v>
-      </c>
-      <c r="H5" s="0" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
@@ -465,24 +390,6 @@
       <c r="B6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="0" t="n">
-        <v>16988</v>
-      </c>
-      <c r="D6" s="0" t="n">
-        <v>17012</v>
-      </c>
-      <c r="E6" s="0" t="n">
-        <v>3012</v>
-      </c>
-      <c r="F6" s="0" t="n">
-        <v>2988</v>
-      </c>
-      <c r="G6" s="0" t="n">
-        <v>0.514079347489372</v>
-      </c>
-      <c r="H6" s="0" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
@@ -491,24 +398,12 @@
       <c r="B7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="4" t="n">
-        <v>17011</v>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>16989</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>2989</v>
-      </c>
-      <c r="F7" s="4" t="n">
-        <v>3011</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>0.504649150939215</v>
-      </c>
-      <c r="H7" s="4" t="n">
-        <v>3</v>
-      </c>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
@@ -517,24 +412,12 @@
       <c r="B8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="4" t="n">
-        <v>17032</v>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>16968</v>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>2968</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>3032</v>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>0.505413048324131</v>
-      </c>
-      <c r="H8" s="4" t="n">
-        <v>4</v>
-      </c>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
@@ -543,24 +426,12 @@
       <c r="B9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="4" t="n">
-        <v>17020</v>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>16980</v>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>2980</v>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>3020</v>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>0.504540154858241</v>
-      </c>
-      <c r="H9" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
@@ -607,7 +478,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.59"/>
   </cols>
@@ -651,84 +522,42 @@
       <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="2" t="n">
-        <v>54.95</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>99.97</v>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>70.92</v>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>99.43</v>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>99.33</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>99.38</v>
-      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="2" t="n">
-        <v>65.77</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>99.91</v>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>79.32</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>95.74</v>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>99.67</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>97.67</v>
-      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="2" t="n">
-        <v>86.52</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>99.71</v>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>92.65</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>99.37</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>99.45</v>
-      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="2" t="n">
-        <v>74.14</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>93.58</v>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>82.74</v>
-      </c>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
@@ -737,15 +566,9 @@
       <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="2" t="n">
-        <v>72.49</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>93.44</v>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>81.65</v>
-      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
@@ -795,7 +618,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.59"/>
   </cols>
@@ -840,84 +663,42 @@
       <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="2" t="n">
-        <v>53.41</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>69.63</v>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>99.23</v>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>99.62</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>99.43</v>
-      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="2" t="n">
-        <v>65.32</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>99.91</v>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>78.99</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>94.9</v>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>99.75</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>97.26</v>
-      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="2" t="n">
-        <v>84.35</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>99.82</v>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>91.44</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>99.14</v>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>99.73</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>99.44</v>
-      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="2" t="n">
-        <v>65.4</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>96.5</v>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>77.96</v>
-      </c>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
@@ -926,15 +707,9 @@
       <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="2" t="n">
-        <v>67.35</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>95.53</v>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>79</v>
-      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
@@ -969,7 +744,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.59"/>
   </cols>
@@ -1014,84 +789,42 @@
       <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="2" t="n">
-        <v>52.07</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>68.48</v>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>98.96</v>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>99.79</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>99.37</v>
-      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="2" t="n">
-        <v>64.62</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>99.98</v>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>78.5</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>94.13</v>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>99.78</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>96.87</v>
-      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="2" t="n">
-        <v>82.65</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>99.82</v>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>90.43</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>98.9</v>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>99.82</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>99.36</v>
-      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="2" t="n">
-        <v>58.61</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>98.02</v>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>73.36</v>
-      </c>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
@@ -1100,15 +833,9 @@
       <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="2" t="n">
-        <v>62.94</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>97.02</v>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>76.34</v>
-      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
@@ -1143,7 +870,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.59"/>
   </cols>
@@ -1188,84 +915,42 @@
       <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="2" t="n">
-        <v>50.92</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>67.48</v>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>98.74</v>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>99.86</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>99.3</v>
-      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="2" t="n">
-        <v>64.08</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>99.98</v>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>78.1</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>93.07</v>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>99.79</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>96.31</v>
-      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="2" t="n">
-        <v>80.27</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>99.87</v>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>89</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>98.51</v>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>99.85</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>99.18</v>
-      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="2" t="n">
-        <v>53.54</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>98.92</v>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>69.48</v>
-      </c>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
@@ -1274,15 +959,9 @@
       <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="2" t="n">
-        <v>60.31</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>98</v>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>74.67</v>
-      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
@@ -1317,7 +996,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G12"/>
-  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.59"/>
   </cols>
@@ -1362,84 +1041,42 @@
       <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="2" t="n">
-        <v>49.59</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>66.31</v>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>98.51</v>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>99.91</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>99.21</v>
-      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="2" t="n">
-        <v>63.07</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>77.35</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>92.15</v>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>99.84</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>95.84</v>
-      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="2" t="n">
-        <v>78.18</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>99.94</v>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>87.73</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>97.93</v>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>99.88</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>98.89</v>
-      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="2" t="n">
-        <v>49.65</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>99.34</v>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>66.21</v>
-      </c>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
@@ -1448,15 +1085,9 @@
       <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="2" t="n">
-        <v>57.82</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>98.9</v>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>72.97</v>
-      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
@@ -1491,7 +1122,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K26"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
@@ -1507,22 +1138,22 @@
         <v>3</v>
       </c>
       <c r="E1" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>22</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>23</v>
       </c>
       <c r="H1" s="6" t="s">
         <v>6</v>
       </c>
       <c r="I1" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J1" s="6" t="s">
         <v>24</v>
-      </c>
-      <c r="J1" s="6" t="s">
-        <v>25</v>
       </c>
       <c r="K1" s="6" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
Fixed for loops in validate and test
</commit_message>
<xml_diff>
--- a/train_results.xlsx
+++ b/train_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hogdo\git\fetch\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E99BDF2-6BC4-4AA6-9709-1AE60B54DA84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40AA443A-0C62-41E6-8D29-77B3AB361408}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12084" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="11148" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Train overview" sheetId="1" r:id="rId1"/>
@@ -171,9 +171,6 @@
   <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -194,6 +191,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -604,36 +604,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C2">
@@ -656,10 +656,10 @@
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C3">
@@ -682,10 +682,10 @@
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C4">
@@ -708,10 +708,10 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C5">
@@ -734,82 +734,160 @@
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="C6">
+        <v>16929</v>
+      </c>
+      <c r="D6">
+        <v>17071</v>
+      </c>
+      <c r="E6">
+        <v>3071</v>
+      </c>
+      <c r="F6">
+        <v>2929</v>
+      </c>
+      <c r="G6">
+        <v>0.54781701120119197</v>
+      </c>
+      <c r="H6">
+        <v>2</v>
+      </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
+      <c r="C7" s="4">
+        <v>17018</v>
+      </c>
+      <c r="D7" s="4">
+        <v>16982</v>
+      </c>
+      <c r="E7" s="4">
+        <v>2982</v>
+      </c>
+      <c r="F7" s="4">
+        <v>3018</v>
+      </c>
+      <c r="G7" s="4">
+        <v>0.50474521943501005</v>
+      </c>
+      <c r="H7" s="4">
+        <v>3</v>
+      </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
+      <c r="C8" s="4">
+        <v>17021</v>
+      </c>
+      <c r="D8" s="4">
+        <v>16979</v>
+      </c>
+      <c r="E8" s="4">
+        <v>2979</v>
+      </c>
+      <c r="F8" s="4">
+        <v>3021</v>
+      </c>
+      <c r="G8" s="4">
+        <v>0.50544260465909496</v>
+      </c>
+      <c r="H8" s="4">
+        <v>3</v>
+      </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
+      <c r="C9" s="4">
+        <v>17008</v>
+      </c>
+      <c r="D9" s="4">
+        <v>16992</v>
+      </c>
+      <c r="E9" s="4">
+        <v>2992</v>
+      </c>
+      <c r="F9" s="4">
+        <v>3008</v>
+      </c>
+      <c r="G9" s="4">
+        <v>0.50408383778163302</v>
+      </c>
+      <c r="H9" s="4">
+        <v>3</v>
+      </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
+      <c r="C10" s="4">
+        <v>16936</v>
+      </c>
+      <c r="D10" s="4">
+        <v>17064</v>
+      </c>
+      <c r="E10" s="4">
+        <v>3064</v>
+      </c>
+      <c r="F10" s="4">
+        <v>2936</v>
+      </c>
+      <c r="G10" s="4">
+        <v>0.50394623856695797</v>
+      </c>
+      <c r="H10" s="4">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
+      <c r="C11" s="4">
+        <v>16982</v>
+      </c>
+      <c r="D11" s="4">
+        <v>17018</v>
+      </c>
+      <c r="E11" s="4">
+        <v>3018</v>
+      </c>
+      <c r="F11" s="4">
+        <v>2982</v>
+      </c>
+      <c r="G11" s="4">
+        <v>0.50643191261897003</v>
+      </c>
+      <c r="H11" s="4">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
@@ -830,142 +908,142 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1" t="s">
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>59.95</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="2">
         <v>98.42</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="2">
         <v>74.510000000000005</v>
       </c>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>67.47</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="2">
         <v>96.96</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <v>79.569999999999993</v>
       </c>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="2">
         <v>62.7</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="2">
         <v>98.1</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="2">
         <v>76.5</v>
       </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="2">
         <v>61.87</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="2">
         <v>77.12</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="2">
         <v>68.66</v>
       </c>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -990,128 +1068,128 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="2"/>
-      <c r="B1" s="1" t="s">
+      <c r="A1" s="1"/>
+      <c r="B1" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1" t="s">
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>58.28</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="2">
         <v>98.88</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="2">
         <v>73.430000000000007</v>
       </c>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>67.02</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="2">
         <v>97.7</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <v>79.5</v>
       </c>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="2">
         <v>61.96</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="2">
         <v>98.66</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="2">
         <v>76.12</v>
       </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="2">
         <v>54.46</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="2">
         <v>83.01</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="2">
         <v>65.77</v>
       </c>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="3"/>
+      <c r="A8" s="2"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="3"/>
+      <c r="A10" s="2"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="3"/>
+      <c r="A12" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1136,128 +1214,128 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="2"/>
-      <c r="B1" s="1" t="s">
+      <c r="A1" s="1"/>
+      <c r="B1" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1" t="s">
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>56.99</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="2">
         <v>99.09</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="2">
         <v>72.36</v>
       </c>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>66.52</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="2">
         <v>98.38</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <v>79.37</v>
       </c>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="2">
         <v>61.16</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="2">
         <v>99.15</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="2">
         <v>76.12</v>
       </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="2">
         <v>47.99</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="2">
         <v>86.9</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="2">
         <v>61.83</v>
       </c>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="3"/>
+      <c r="A8" s="2"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="3"/>
+      <c r="A10" s="2"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="3"/>
+      <c r="A12" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1282,128 +1360,128 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="2"/>
-      <c r="B1" s="1" t="s">
+      <c r="A1" s="1"/>
+      <c r="B1" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1" t="s">
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>55.55</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="2">
         <v>99.33</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="2">
         <v>71.25</v>
       </c>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>65.88</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="2">
         <v>98.7</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <v>79.010000000000005</v>
       </c>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="2">
         <v>60.23</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="2">
         <v>99.48</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="2">
         <v>75.040000000000006</v>
       </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="2">
         <v>44.48</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="2">
         <v>91.03</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="2">
         <v>59.76</v>
       </c>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="3"/>
+      <c r="A8" s="2"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="3"/>
+      <c r="A10" s="2"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="3"/>
+      <c r="A12" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1428,128 +1506,128 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="2"/>
-      <c r="B1" s="1" t="s">
+      <c r="A1" s="1"/>
+      <c r="B1" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1" t="s">
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>54.19</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="2">
         <v>99.59</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="2">
         <v>70.180000000000007</v>
       </c>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>64.78</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="2">
         <v>99.04</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <v>78.33</v>
       </c>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="2">
         <v>59.24</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="2">
         <v>99.62</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="2">
         <v>74.3</v>
       </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="2">
         <v>42.99</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="2">
         <v>94.43</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="2">
         <v>59.08</v>
       </c>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="3"/>
+      <c r="A8" s="2"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="3"/>
+      <c r="A10" s="2"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="3"/>
+      <c r="A12" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1571,464 +1649,464 @@
   <sheetFormatPr defaultColWidth="11.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="5" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="7"/>
-      <c r="K6" s="7"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="6"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="6"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="8"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
-      <c r="K8" s="8"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="7"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
-      <c r="K9" s="8"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="7"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8"/>
-      <c r="K10" s="8"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="9" t="s">
+      <c r="A11" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-      <c r="K11" s="9"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="8"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+      <c r="K14" s="2"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
-      <c r="H16" s="7"/>
-      <c r="I16" s="7"/>
-      <c r="J16" s="7"/>
-      <c r="K16" s="7"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6"/>
+      <c r="H16" s="6"/>
+      <c r="I16" s="6"/>
+      <c r="J16" s="6"/>
+      <c r="K16" s="6"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="8"/>
-      <c r="I17" s="8"/>
-      <c r="J17" s="8"/>
-      <c r="K17" s="8"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="7"/>
+      <c r="J17" s="7"/>
+      <c r="K17" s="7"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" s="8" t="s">
+      <c r="A18" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B18" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
-      <c r="I18" s="8"/>
-      <c r="J18" s="8"/>
-      <c r="K18" s="8"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="7"/>
+      <c r="I18" s="7"/>
+      <c r="J18" s="7"/>
+      <c r="K18" s="7"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
-      <c r="J19" s="8"/>
-      <c r="K19" s="8"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="7"/>
+      <c r="J19" s="7"/>
+      <c r="K19" s="7"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" s="8" t="s">
+      <c r="A20" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="B20" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="8"/>
-      <c r="K20" s="8"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="7"/>
+      <c r="H20" s="7"/>
+      <c r="I20" s="7"/>
+      <c r="J20" s="7"/>
+      <c r="K20" s="7"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" s="9" t="s">
+      <c r="A21" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C21" s="9"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
-      <c r="G21" s="9"/>
-      <c r="H21" s="9"/>
-      <c r="I21" s="9"/>
-      <c r="J21" s="9"/>
-      <c r="K21" s="9"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="8"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="8"/>
+      <c r="J21" s="8"/>
+      <c r="K21" s="8"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
-      <c r="I22" s="3"/>
-      <c r="J22" s="3"/>
-      <c r="K22" s="3"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
+      <c r="J22" s="2"/>
+      <c r="K22" s="2"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
-      <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
-      <c r="I23" s="3"/>
-      <c r="J23" s="3"/>
-      <c r="K23" s="3"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
+      <c r="J23" s="2"/>
+      <c r="K23" s="2"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
-      <c r="G24" s="3"/>
-      <c r="H24" s="3"/>
-      <c r="I24" s="3"/>
-      <c r="J24" s="3"/>
-      <c r="K24" s="3"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
+      <c r="A25" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
-      <c r="E25" s="3"/>
-      <c r="F25" s="3"/>
-      <c r="G25" s="3"/>
-      <c r="H25" s="3"/>
-      <c r="I25" s="3"/>
-      <c r="J25" s="3"/>
-      <c r="K25" s="3"/>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
+      <c r="J25" s="2"/>
+      <c r="K25" s="2"/>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A26" s="7" t="s">
+      <c r="A26" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="7"/>
-      <c r="F26" s="7"/>
-      <c r="G26" s="7"/>
-      <c r="H26" s="7"/>
-      <c r="I26" s="7"/>
-      <c r="J26" s="7"/>
-      <c r="K26" s="7"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="6"/>
+      <c r="H26" s="6"/>
+      <c r="I26" s="6"/>
+      <c r="J26" s="6"/>
+      <c r="K26" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>

</xml_diff>